<commit_message>
Iniziato export Fidente, fatto export Lampo, modificato export Sogedi, inserita data cambio qualidica per i manutentori komplett, modifica API richiesta ferie permessi, inserito codice commessa come campo obbligatorio tramite personalizzazione, impostato che se si
cancella una timbratura con attività cancella anche quella,
</commit_message>
<xml_diff>
--- a/PowerWeb/ExcelModels/ExportFatturato.xlsx
+++ b/PowerWeb/ExcelModels/ExportFatturato.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29426"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\backup\PWNuovo\PowerWeb\ExcelModels\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7E8168CF-EBC7-4CBF-A781-4E61F6B6D0E8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{42256620-1105-46A4-8EA8-1903F30A5A75}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Foglio1" sheetId="1" r:id="rId1"/>
@@ -113,7 +113,18 @@
   <cellStyles count="1">
     <cellStyle name="Normale" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="1">
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -393,6 +404,7 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="15.140625" customWidth="1"/>
+    <col min="2" max="2" width="36.5703125" customWidth="1"/>
     <col min="3" max="3" width="14.85546875" customWidth="1"/>
     <col min="4" max="4" width="22.5703125" customWidth="1"/>
     <col min="5" max="5" width="21.140625" customWidth="1"/>
@@ -421,6 +433,11 @@
     </row>
   </sheetData>
   <autoFilter ref="B1" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
+  <conditionalFormatting sqref="F1:F1048576">
+    <cfRule type="cellIs" dxfId="0" priority="1" operator="lessThan">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>